<commit_message>
feat: keep one HTML report per run; run CRT-050 on Chromium only
- Local runs write reports/html/test_report_<yyyyMMdd_HHmmss>/; the newest
  10 are kept (REPORT_HISTORY). npm run report opens the latest or a given run.
- CRT-050 is tagged @chromium-only and left out of Firefox/WebKit instead of
  being skipped there.
- README: remove the contributor conventions and roadmap sections.
</commit_message>
<xml_diff>
--- a/docs/DemoBlaze_Test_Cases.xlsx
+++ b/docs/DemoBlaze_Test_Cases.xlsx
@@ -337,7 +337,7 @@
     <t xml:space="preserve">1.7</t>
   </si>
   <si>
-    <t xml:space="preserve">Root causes of the latest run's 5 failures: new defect PD-28 (bought items stay in the cart when OK is pressed quickly), covered by CRT-050; LGN-005 starts on Home to avoid the shared guest cart; the performance check runs on its own and uses the median of 3 cold loads.</t>
+    <t xml:space="preserve">Root causes of the latest run's 5 failures: new defect PD-28 (bought items stay in the cart when OK is pressed quickly), covered by CRT-050; LGN-005 starts on Home to avoid the shared guest cart; the performance check runs on its own and uses the median of 3 cold loads. Confirmed by the next full run: 167 passed, 0 failed, 0 flaky.</t>
   </si>
   <si>
     <t xml:space="preserve">TC ID</t>
@@ -4685,7 +4685,7 @@
       <c r="G68" s="11"/>
       <c r="H68" s="11"/>
     </row>
-    <row r="69" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="81" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="s">
         <v>101</v>
       </c>

</xml_diff>

<commit_message>
docs: renumber potential defects after withdrawing PD-14
PD-15..PD-28 become PD-14..PD-27 in the workbook, the defect register, the
@pd-xx test tags, code comments and the README.
</commit_message>
<xml_diff>
--- a/docs/DemoBlaze_Test_Cases.xlsx
+++ b/docs/DemoBlaze_Test_Cases.xlsx
@@ -450,7 +450,7 @@
     <t xml:space="preserve">Page reloads on cart.html, shows 'Welcome {VALID_USER}' and lists {VALID_USER}'s cart item.</t>
   </si>
   <si>
-    <t xml:space="preserve">Page reloaded on cart.html with 'Welcome &lt;user&gt;' and the user's cart item listed. (The journey starts on Home: opening cart.html directly as a guest loads the shared guest cart (PD-22), hundreds of items, which once slowed the API enough to time the test out.)</t>
+    <t xml:space="preserve">Page reloaded on cart.html with 'Welcome &lt;user&gt;' and the user's cart item listed. (The journey starts on Home: opening cart.html directly as a guest loads the shared guest cart (PD-21), hundreds of items, which once slowed the API enough to time the test out.)</t>
   </si>
   <si>
     <t xml:space="preserve">LGN-006</t>
@@ -598,10 +598,10 @@
     <t xml:space="preserve">Login succeeds and the navbar shows 'Welcome {VALID_USER}' (no spaces).</t>
   </si>
   <si>
-    <t xml:space="preserve">Fails as expected (PD-26): ' &lt;username&gt; ' with spaces gave 'User does not exist.'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD-26</t>
+    <t xml:space="preserve">Fails as expected (PD-25): ' &lt;username&gt; ' with spaces gave 'User does not exist.'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD-25</t>
   </si>
   <si>
     <t xml:space="preserve">LGN-013</t>
@@ -623,10 +623,10 @@
     <t xml:space="preserve">Login succeeds and the navbar shows 'Welcome {VALID_USER}'.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fails as expected (PD-27): username in upper case gave 'User does not exist.'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD-27</t>
+    <t xml:space="preserve">Fails as expected (PD-26): username in upper case gave 'User does not exist.'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD-26</t>
   </si>
   <si>
     <t xml:space="preserve">LGN-014</t>
@@ -778,10 +778,10 @@
     <t xml:space="preserve">After the configured threshold (e.g. 5 attempts, to confirm with PO), further attempts are blocked with a lockout, CAPTCHA or rate-limit message.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fails as expected (PD-25): the 10th consecutive wrong password still returned 'Wrong password.' – no lockout or rate limit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD-25</t>
+    <t xml:space="preserve">Fails as expected (PD-24): the 10th consecutive wrong password still returned 'Wrong password.' – no lockout or rate limit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD-24</t>
   </si>
   <si>
     <t xml:space="preserve">LGN-019</t>
@@ -798,10 +798,10 @@
     <t xml:space="preserve">User is logged in ('Welcome {VALID_USER}'). Only one POST /login request is sent; no error alert.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fails as expected (PD-23): double-click sent two POST /login requests.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD-23</t>
+    <t xml:space="preserve">Fails as expected (PD-22): double-click sent two POST /login requests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD-22</t>
   </si>
   <si>
     <t xml:space="preserve">LGN-020</t>
@@ -957,10 +957,10 @@
     <t xml:space="preserve">The token is random and opaque; decoding it does not reveal the username or any predictable value.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fails as expected (PD-18): token decodes to username + number.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD-18</t>
+    <t xml:space="preserve">Fails as expected (PD-17): token decodes to username + number.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD-17</t>
   </si>
   <si>
     <t xml:space="preserve">tests/security/session-security.spec.ts</t>
@@ -1119,10 +1119,10 @@
     <t xml:space="preserve">HTTP 401 Unauthorized.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fails as expected (PD-19): HTTP 200 + errorMessage instead of 401.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD-19</t>
+    <t xml:space="preserve">Fails as expected (PD-18): HTTP 200 + errorMessage instead of 401.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD-18</t>
   </si>
   <si>
     <t xml:space="preserve">CRT-001</t>
@@ -1194,7 +1194,7 @@
     <t xml:space="preserve">Page showed 'undefined $undefined' with an active 'Add to cart'; clicking it gave alert 'Bad parameter, token malformed.'</t>
   </si>
   <si>
-    <t xml:space="preserve">PD-15</t>
+    <t xml:space="preserve">PD-14</t>
   </si>
   <si>
     <t xml:space="preserve">CRT-004</t>
@@ -1213,7 +1213,7 @@
     <t xml:space="preserve">Blank product area; Console: Uncaught TypeError: Cannot read properties of undefined (reading 'split') at prod.js:39.</t>
   </si>
   <si>
-    <t xml:space="preserve">PD-16</t>
+    <t xml:space="preserve">PD-15</t>
   </si>
   <si>
     <t xml:space="preserve">Console-error judgement – manual (automatable later)</t>
@@ -1738,7 +1738,7 @@
     <t xml:space="preserve">The cart table has no rows, and the server-side cart (/viewcart) is empty.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cart empty on the server and in the UI after purchase. One run failed on Chromium and Firefox because the script pressed OK before the site's cart-clear call had finished: logged as PD-28 (CRT-050). The script now waits for that call, as a user reading the receipt would.</t>
+    <t xml:space="preserve">Cart empty on the server and in the UI after purchase. One run failed on Chromium and Firefox because the script pressed OK before the site's cart-clear call had finished: logged as PD-27 (CRT-050). The script now waits for that call, as a user reading the receipt would.</t>
   </si>
   <si>
     <t xml:space="preserve">CRT-027</t>
@@ -1840,7 +1840,7 @@
     <t xml:space="preserve">Item was purchased and removed from the cart, but confirmation showed 'Amount: 0 USD'.</t>
   </si>
   <si>
-    <t xml:space="preserve">PD-20</t>
+    <t xml:space="preserve">PD-19</t>
   </si>
   <si>
     <t xml:space="preserve">CRT-031</t>
@@ -2085,7 +2085,7 @@
     <t xml:space="preserve">Order placed; the 500-character Name overflowed the dialog horizontally.</t>
   </si>
   <si>
-    <t xml:space="preserve">PD-21</t>
+    <t xml:space="preserve">PD-20</t>
   </si>
   <si>
     <t xml:space="preserve">Visual layout check – manual or visual-regression tool</t>
@@ -2137,10 +2137,10 @@
     <t xml:space="preserve">Exactly one confirmation (one order Id) is shown.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fails as expected (PD-24): double-click sent two order submissions (POST /deletecart twice).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD-24</t>
+    <t xml:space="preserve">Fails as expected (PD-23): double-click sent two order submissions (POST /deletecart twice).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD-23</t>
   </si>
   <si>
     <t xml:space="preserve">CRT-044</t>
@@ -2164,7 +2164,7 @@
     <t xml:space="preserve">Credit card is a plain text input; full number visible while typing.</t>
   </si>
   <si>
-    <t xml:space="preserve">PD-17</t>
+    <t xml:space="preserve">PD-16</t>
   </si>
   <si>
     <t xml:space="preserve">Security UX, assumed requirement – manual</t>
@@ -2249,7 +2249,7 @@
     <t xml:space="preserve">HTTP 404 Not Found.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fails as expected (PD-19): HTTP 200 + 'Not found.' instead of 404.</t>
+    <t xml:space="preserve">Fails as expected (PD-18): HTTP 200 + 'Not found.' instead of 404.</t>
   </si>
   <si>
     <t xml:space="preserve">tests/api/product.api.spec.ts</t>
@@ -2272,10 +2272,10 @@
     <t xml:space="preserve">The cart contains only the one 'Nokia lumia 1520' just added (the guest has a private cart keyed by a unique guest id).</t>
   </si>
   <si>
-    <t xml:space="preserve">Fails as expected (PD-22): /addtocart sent with an empty guest id; the shared cart held 121-134 items from other guests.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD-22</t>
+    <t xml:space="preserve">Fails as expected (PD-21): /addtocart sent with an empty guest id; the shared cart held 121-134 items from other guests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD-21</t>
   </si>
   <si>
     <t xml:space="preserve">CRT-050</t>
@@ -2298,13 +2298,13 @@
     <t xml:space="preserve">The cart is empty, however quickly 'OK' is clicked.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fails as expected (PD-28). First seen in the 20-Oct full run (CRT-026, Chromium and Firefox): OK was pressed about 1 s after Purchase, the move to Home cancelled POST /deletecart (no response), and the server cart still held the item 20 s later. The test reproduces it on demand by slowing that one request down.</t>
+    <t xml:space="preserve">Fails as expected (PD-27). First seen in the 20-Oct full run (CRT-026, Chromium and Firefox): OK was pressed about 1 s after Purchase, the move to Home cancelled POST /deletecart (no response), and the server cart still held the item 20 s later. The test reproduces it on demand by slowing that one request down.</t>
   </si>
   <si>
     <t xml:space="preserve">Automated: Chromium</t>
   </si>
   <si>
-    <t xml:space="preserve">PD-28</t>
+    <t xml:space="preserve">PD-27</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -2659,7 +2659,7 @@
     <t xml:space="preserve">'cWFfc3lfMDExNzkzMDEx' decodes to 'qa_sy_011793011' (username + number). A token for another user could potentially be built without their password (not attempted).</t>
   </si>
   <si>
-    <t xml:space="preserve">reports/evidence/PD-18_LGN-026_&lt;browser&gt;.txt (API log)
+    <t xml:space="preserve">reports/evidence/PD-17_LGN-026_&lt;browser&gt;.txt (API log)
 (&lt;browser&gt; = chromium, firefox, webkit)</t>
   </si>
   <si>
@@ -2683,8 +2683,8 @@
     <t xml:space="preserve">HTTP 200 with {"errorMessage": ...} in the body.</t>
   </si>
   <si>
-    <t xml:space="preserve">reports/evidence/PD-19_LGN-034_api.txt (API log)
-reports/evidence/PD-19_CRT-048_api.txt (API log)</t>
+    <t xml:space="preserve">reports/evidence/PD-18_LGN-034_api.txt (API log)
+reports/evidence/PD-18_CRT-048_api.txt (API log)</t>
   </si>
   <si>
     <t xml:space="preserve">Order amount uses a stale client-side total</t>
@@ -2732,7 +2732,7 @@
     <t xml:space="preserve">Only the Home page creates the guest id cookie ('user'). A guest who lands on a product page first (search result, shared link) sends an empty id, so all such guests read and write the same cart: our test saw 121-134 items from other people. Privacy issue: one guest can see, and buy, another guest's items. Reproduced 20-Oct-2026 by the automated run on Chromium, Firefox and WebKit.</t>
   </si>
   <si>
-    <t xml:space="preserve">reports/evidence/PD-22_CRT-049_&lt;browser&gt;.png + .webm
+    <t xml:space="preserve">reports/evidence/PD-21_CRT-049_&lt;browser&gt;.png + .webm
 (&lt;browser&gt; = chromium, firefox, webkit)</t>
   </si>
   <si>
@@ -2751,7 +2751,7 @@
     <t xml:space="preserve">A double-click calls logIn() twice and sends two POST /login requests. Reproduced 20-Oct-2026 by the automated run (Chromium, Firefox, WebKit).</t>
   </si>
   <si>
-    <t xml:space="preserve">reports/evidence/PD-23_LGN-019_&lt;browser&gt;.png + .webm
+    <t xml:space="preserve">reports/evidence/PD-22_LGN-019_&lt;browser&gt;.png + .webm
 (&lt;browser&gt; = chromium, firefox, webkit)</t>
   </si>
   <si>
@@ -2771,7 +2771,7 @@
     <t xml:space="preserve">A double-click runs purchaseOrder() twice: two order submissions (POST /deletecart twice) and the confirmation is regenerated. Reproduced 20-Oct-2026 by the automated run (Chromium, Firefox, WebKit).</t>
   </si>
   <si>
-    <t xml:space="preserve">reports/evidence/PD-24_CRT-043_&lt;browser&gt;.png + .webm
+    <t xml:space="preserve">reports/evidence/PD-23_CRT-043_&lt;browser&gt;.png + .webm
 (&lt;browser&gt; = chromium, firefox, webkit)</t>
   </si>
   <si>
@@ -2792,7 +2792,7 @@
     <t xml:space="preserve">10 consecutive wrong passwords all returned 'Wrong password.'; nothing slows down or blocks guessing, so passwords can be brute-forced. Reproduced 20-Oct-2026 by the automated run (Chromium, Firefox, WebKit).</t>
   </si>
   <si>
-    <t xml:space="preserve">reports/evidence/PD-25_LGN-018_&lt;browser&gt;.png + .webm
+    <t xml:space="preserve">reports/evidence/PD-24_LGN-018_&lt;browser&gt;.png + .webm
 (&lt;browser&gt; = chromium, firefox, webkit)</t>
   </si>
   <si>
@@ -2810,7 +2810,7 @@
     <t xml:space="preserve">' &lt;username&gt; ' with surrounding spaces returns 'User does not exist.' Reproduced 20-Oct-2026 by the automated run (Chromium, Firefox, WebKit).</t>
   </si>
   <si>
-    <t xml:space="preserve">reports/evidence/PD-26_LGN-012_&lt;browser&gt;.png + .webm
+    <t xml:space="preserve">reports/evidence/PD-25_LGN-012_&lt;browser&gt;.png + .webm
 (&lt;browser&gt; = chromium, firefox, webkit)</t>
   </si>
   <si>
@@ -2828,7 +2828,7 @@
     <t xml:space="preserve">The username in upper case returns 'User does not exist.' Reproduced 20-Oct-2026 by the automated run (Chromium, Firefox, WebKit).</t>
   </si>
   <si>
-    <t xml:space="preserve">reports/evidence/PD-27_LGN-013_&lt;browser&gt;.png + .webm
+    <t xml:space="preserve">reports/evidence/PD-26_LGN-013_&lt;browser&gt;.png + .webm
 (&lt;browser&gt; = chromium, firefox, webkit)</t>
   </si>
   <si>
@@ -2851,7 +2851,7 @@
     <t xml:space="preserve">purchaseOrder() sends POST /deletecart without waiting for it, and OK goes to Home straight away. If OK is pressed before that request finishes, the browser cancels it and the server cart keeps the purchased items (automated run: the item was still there 20 s later). The customer can then pay for the same items again. Found by the automated run on 20-Oct-2026 (Chromium, Firefox).</t>
   </si>
   <si>
-    <t xml:space="preserve">reports/evidence/PD-28_CRT-050_chromium.png + .webm</t>
+    <t xml:space="preserve">reports/evidence/PD-27_CRT-050_chromium.png + .webm</t>
   </si>
   <si>
     <t xml:space="preserve">Note: DemoBlaze has no published requirements. 'Expected' follows common e-commerce practice, so 'Potential defect – requirement to confirm' items should be agreed with the product owner before being raised as bugs. 'Reproduced?' = observed when the related test was run on 19-Oct-2026.</t>

</xml_diff>